<commit_message>
updated w/ Mmatrix, some CEATTLE
</commit_message>
<xml_diff>
--- a/runs/ceattle/BSP0.xlsx
+++ b/runs/ceattle/BSP0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jim/_mymods/noaa-afsc/EBS_pollock/runs/ceattle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E750070-AF8E-BE42-BD33-DBC59D17FBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8652FDA9-C2DB-3447-A3A7-63D39EADC562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="-21100" windowWidth="34560" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26077,18 +26077,18 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -26114,67 +26114,67 @@
         <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
@@ -26200,17 +26200,17 @@
         <v>9</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
         <v>0.7</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
       <c r="L2">
         <v>1</v>
       </c>
@@ -26230,34 +26230,34 @@
         <v>1</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T2">
         <v>0</v>
       </c>
       <c r="U2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2">
         <v>0</v>
       </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
       <c r="X2">
         <v>0</v>
       </c>
-      <c r="Y2">
-        <v>1</v>
-      </c>
       <c r="Z2">
         <v>0</v>
       </c>
       <c r="AA2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AB2">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -26280,16 +26280,13 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3">
         <v>2</v>
@@ -26304,37 +26301,40 @@
         <v>1</v>
       </c>
       <c r="P3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q3">
         <v>1</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
       <c r="U3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3">
         <v>0</v>
       </c>
+      <c r="W3">
+        <v>1</v>
+      </c>
       <c r="X3">
         <v>0</v>
       </c>
-      <c r="Y3">
-        <v>1</v>
-      </c>
       <c r="Z3">
         <v>0</v>
       </c>
       <c r="AA3">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -26357,19 +26357,16 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
         <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>3</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -26381,37 +26378,40 @@
         <v>1</v>
       </c>
       <c r="P4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4">
         <v>0</v>
       </c>
       <c r="U4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V4">
         <v>0</v>
       </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
       <c r="X4">
         <v>0</v>
       </c>
-      <c r="Y4">
-        <v>1</v>
-      </c>
       <c r="Z4">
         <v>0</v>
       </c>
       <c r="AA4">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -26434,19 +26434,16 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
         <v>2</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>4</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -26458,37 +26455,40 @@
         <v>1</v>
       </c>
       <c r="P5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q5">
         <v>1</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5">
         <v>0</v>
       </c>
       <c r="U5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V5">
         <v>0</v>
       </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
       <c r="X5">
         <v>0</v>
       </c>
-      <c r="Y5">
-        <v>1</v>
-      </c>
       <c r="Z5">
         <v>0</v>
       </c>
       <c r="AA5">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -26511,61 +26511,61 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
         <v>2</v>
       </c>
-      <c r="L6">
+      <c r="N6">
         <v>4</v>
       </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
         <v>5</v>
       </c>
-      <c r="O6">
-        <v>1</v>
-      </c>
-      <c r="P6">
-        <v>1</v>
-      </c>
       <c r="Q6">
         <v>1</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6">
         <v>0</v>
       </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
       <c r="X6">
         <v>0</v>
       </c>
-      <c r="Y6">
-        <v>1</v>
-      </c>
       <c r="Z6">
         <v>0</v>
       </c>
       <c r="AA6">
         <v>1</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.2">
@@ -26588,61 +26588,61 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <v>2</v>
       </c>
-      <c r="L7">
+      <c r="N7">
         <v>4</v>
       </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-      <c r="N7">
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
         <v>6</v>
       </c>
-      <c r="O7">
-        <v>1</v>
-      </c>
-      <c r="P7">
-        <v>1</v>
-      </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7">
         <v>0</v>
       </c>
       <c r="U7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V7">
         <v>0</v>
       </c>
+      <c r="W7">
+        <v>1</v>
+      </c>
       <c r="X7">
         <v>0</v>
       </c>
-      <c r="Y7">
-        <v>1</v>
-      </c>
       <c r="Z7">
         <v>0</v>
       </c>
       <c r="AA7">
         <v>1</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>